<commit_message>
Add Moneyball Auction Assistant
</commit_message>
<xml_diff>
--- a/AuctionWorkBook.xlsx
+++ b/AuctionWorkBook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hp\Documents\Projects\MoneyBall2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DD93A04-D94E-486D-80F5-A440A34847CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3469FFD8-5340-4380-A941-E34013FEADF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{19692BFB-9572-4592-AF0C-699A45FCFCB8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3883" uniqueCount="1008">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3899" uniqueCount="1021">
   <si>
     <t>S.no</t>
   </si>
@@ -3073,9 +3073,6 @@
     <t>Squad Status</t>
   </si>
   <si>
-    <t>me</t>
-  </si>
-  <si>
     <t>Player ID</t>
   </si>
   <si>
@@ -3083,13 +3080,55 @@
   </si>
   <si>
     <t xml:space="preserve">Team: </t>
+  </si>
+  <si>
+    <t>mess</t>
+  </si>
+  <si>
+    <t>Position Role</t>
+  </si>
+  <si>
+    <t>Drafted</t>
+  </si>
+  <si>
+    <t>Min Requirement</t>
+  </si>
+  <si>
+    <t>Min Needed</t>
+  </si>
+  <si>
+    <t>Max Cap</t>
+  </si>
+  <si>
+    <t>Max Extra</t>
+  </si>
+  <si>
+    <t>Forwards (FW)</t>
+  </si>
+  <si>
+    <t>Midfielders (MF)</t>
+  </si>
+  <si>
+    <t>Defenders (DF)</t>
+  </si>
+  <si>
+    <t>Goalkeepers (GK)</t>
+  </si>
+  <si>
+    <t>TOTAL SQUAD</t>
+  </si>
+  <si>
+    <t>Remaining</t>
+  </si>
+  <si>
+    <t>Total Roster</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3140,8 +3179,16 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3181,6 +3228,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF333333"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD3D3D3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3227,7 +3292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -3245,14 +3310,149 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFD3D3D3"/>
+      <color rgb="FF333333"/>
       <color rgb="FF00FF00"/>
     </mruColors>
   </colors>
@@ -60124,7 +60324,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3F22BC2-839C-4E62-BE00-402DF1C1F3A9}">
-  <dimension ref="A1:N310"/>
+  <dimension ref="A1:E310"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -60136,108 +60336,30 @@
     <col min="7" max="7" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" ht="19.5" thickBot="1">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="19.5" thickBot="1">
       <c r="A1" s="2" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="5" customFormat="1" ht="18.75">
+      <c r="A2" s="5" cm="1">
+        <f t="array" ref="A2">IF($B$1="", "", IFERROR(TRANSPOSE(_xlfn._xlws.FILTER(Master_List!$A$2:$A$200, ISNUMBER(SEARCH($B$1, Master_List!$B$2:$B$200)))), ""))</f>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="6" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A3" s="6" t="str" cm="1">
+        <f t="array" ref="A3">IF($B$1="", "", IFERROR(TRANSPOSE(_xlfn._xlws.FILTER(Master_List!$B$2:$B$200, ISNUMBER(SEARCH($B$1, Master_List!$B$2:$B$200)))), ""))</f>
+        <v>Lionel Messi</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="3" customFormat="1"/>
+    <row r="5" spans="1:5" s="7" customFormat="1" ht="15.75">
+      <c r="A5" s="7" t="s">
         <v>1004</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" s="5" customFormat="1" ht="18.75">
-      <c r="A2" s="5" cm="1">
-        <f t="array" ref="A2:N2">IF($B$1="", "", IFERROR(TRANSPOSE(_xlfn._xlws.FILTER(Master_List!$A$2:$A$200, ISNUMBER(SEARCH($B$1, Master_List!$B$2:$B$200)))), ""))</f>
-        <v>23</v>
-      </c>
-      <c r="B2" s="5">
-        <v>69</v>
-      </c>
-      <c r="C2" s="5">
-        <v>84</v>
-      </c>
-      <c r="D2" s="5">
-        <v>86</v>
-      </c>
-      <c r="E2" s="5">
-        <v>99</v>
-      </c>
-      <c r="F2" s="5">
-        <v>102</v>
-      </c>
-      <c r="G2" s="5">
-        <v>153</v>
-      </c>
-      <c r="H2" s="5">
-        <v>159</v>
-      </c>
-      <c r="I2" s="5">
-        <v>161</v>
-      </c>
-      <c r="J2" s="5">
-        <v>163</v>
-      </c>
-      <c r="K2" s="5">
-        <v>166</v>
-      </c>
-      <c r="L2" s="5">
-        <v>167</v>
-      </c>
-      <c r="M2" s="5">
-        <v>192</v>
-      </c>
-      <c r="N2" s="5">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" s="6" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A3" s="6" t="str" cm="1">
-        <f t="array" ref="A3:N3">IF($B$1="", "", IFERROR(TRANSPOSE(_xlfn._xlws.FILTER(Master_List!$B$2:$B$200, ISNUMBER(SEARCH($B$1, Master_List!$B$2:$B$200)))), ""))</f>
-        <v>James Maddison</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Yan Sommer</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Lionel Messi</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <v>Mohamed Salah</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Romelu Lukaku</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Memphis Depay</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Mats Hummels</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Reece James</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Upamecano</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Ferland Mendy</v>
-      </c>
-      <c r="K3" s="6" t="str">
-        <v>Cristian Romero</v>
-      </c>
-      <c r="L3" s="6" t="str">
-        <v>Gimenez</v>
-      </c>
-      <c r="M3" s="6" t="str">
-        <v>Nicolas Otamendi</v>
-      </c>
-      <c r="N3" s="6" t="str">
-        <v>Bremer</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" s="3" customFormat="1"/>
-    <row r="5" spans="1:14" s="7" customFormat="1" ht="15.75">
-      <c r="A5" s="7" t="s">
-        <v>1005</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>983</v>
@@ -60252,7 +60374,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:5">
       <c r="B6" t="str">
         <f>IF(A6="","", _xlfn.XLOOKUP(A6, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60262,7 +60384,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:5">
       <c r="B7" t="str">
         <f>IF(A7="","", _xlfn.XLOOKUP(A7, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60272,7 +60394,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:5">
       <c r="B8" t="str">
         <f>IF(A8="","", _xlfn.XLOOKUP(A8, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60282,7 +60404,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:5">
       <c r="B9" t="str">
         <f>IF(A9="","", _xlfn.XLOOKUP(A9, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60292,7 +60414,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:5">
       <c r="B10" t="str">
         <f>IF(A10="","", _xlfn.XLOOKUP(A10, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60302,7 +60424,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:5">
       <c r="B11" t="str">
         <f>IF(A11="","", _xlfn.XLOOKUP(A11, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60312,7 +60434,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:5">
       <c r="B12" t="str">
         <f>IF(A12="","", _xlfn.XLOOKUP(A12, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60322,7 +60444,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:5">
       <c r="B13" t="str">
         <f>IF(A13="","", _xlfn.XLOOKUP(A13, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60332,7 +60454,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:5">
       <c r="B14" t="str">
         <f>IF(A14="","", _xlfn.XLOOKUP(A14, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60342,7 +60464,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:5">
       <c r="B15" t="str">
         <f>IF(A15="","", _xlfn.XLOOKUP(A15, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -60352,7 +60474,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:5">
       <c r="B16" t="str">
         <f>IF(A16="","", _xlfn.XLOOKUP(A16, Master_List!A:A, Master_List!B:B, "Invalid ID"))</f>
         <v/>
@@ -63784,49 +63906,213 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B5C1983-FBE2-43BE-AF5A-C06BDFD418C3}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="4" max="6" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B1">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="str">
+    <row r="2" spans="1:6" s="11" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A2" s="11" t="s">
+        <v>998</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>999</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="10" customFormat="1" ht="29.25" customHeight="1">
+      <c r="A3" s="10" t="str">
         <f>_xlfn.XLOOKUP(B1, Dashboard!A2:A11, Dashboard!B2:B11, "Team " &amp; B1)</f>
         <v>A</v>
       </c>
-      <c r="B2">
+      <c r="B3" s="10">
+        <f>_xlfn.XLOOKUP(B1, Dashboard!A2:A11, Dashboard!C2:C11, 0)</f>
+        <v>900</v>
+      </c>
+      <c r="C3" s="10">
+        <f>_xlfn.XLOOKUP(B1, Dashboard!A2:A11, Dashboard!D2:D11, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="10">
         <f>_xlfn.XLOOKUP(B1, Dashboard!A2:A11, Dashboard!E2:E11, 0)</f>
         <v>900</v>
       </c>
-      <c r="C2" t="str">
+      <c r="E3" s="10" t="str">
         <f>_xlfn.XLOOKUP(B1, Dashboard!A2:A11, Dashboard!F2:F11, 0) &amp; " / 16"</f>
         <v>0 / 16</v>
       </c>
-      <c r="D2" s="8">
-        <f>16 - _xlfn.XLOOKUP(B1, Dashboard!A2:A11, Dashboard!F2:F11, 0)</f>
+    </row>
+    <row r="4" spans="1:6" s="9" customFormat="1" ht="25.5" customHeight="1">
+      <c r="A4" s="9" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>1010</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>1011</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B5">
+        <f>COUNTIFS(Auction_Log!D5:D200, B1, Auction_Log!C5:C200, "Forwards")</f>
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <f>MAX(0, 2 - B5)</f>
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <f>MAX(0, 4 - B5)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B6">
+        <f>COUNTIFS(Auction_Log!D5:D200, B1, Auction_Log!C5:C200, "Midfield")</f>
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <f>MAX(0, 2 - B6)</f>
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <f>MAX(0, 5 - B6)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B7">
+        <f>COUNTIFS(Auction_Log!D5:D200, B1, Auction_Log!C5:C200, "Defender")</f>
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <f>MAX(0, 3 - B7)</f>
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <f>MAX(0, 5 - B7)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B8">
+        <f>COUNTIFS(Auction_Log!D5:D200, B1, Auction_Log!C5:C200, "Goalkeeper")</f>
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <f>MAX(0, 1 - B8)</f>
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <f>MAX(0, 2 - B8)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B9" s="8">
+        <f>SUM(B5:B8)</f>
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <f>SUM(D5:D8)</f>
+        <v>8</v>
+      </c>
+      <c r="E9">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="B3">
-        <f>B2 - ((11 - _xlfn.XLOOKUP(B1, Dashboard!A2:A11, Dashboard!F2:F11, 0)) * 1)</f>
-        <v>889</v>
-      </c>
-      <c r="D3">
-        <f>IF(D2=0, 0, ROUND(B2 / D2, 1))</f>
-        <v>56.3</v>
+      <c r="F9">
+        <f>16 - B9</f>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F5:F8">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:F8">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D5:D8">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>